<commit_message>
Added live weight of lost animals for layers + slaughter weight for hens
</commit_message>
<xml_diff>
--- a/data/default/LayerHerd.xlsx
+++ b/data/default/LayerHerd.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="136">
   <si>
     <t>value</t>
   </si>
@@ -404,9 +404,6 @@
     <t>share_in_ration</t>
   </si>
   <si>
-    <t>Creates problems with too much poultry meat</t>
-  </si>
-  <si>
     <t>Slaughter and live weights</t>
   </si>
   <si>
@@ -437,9 +434,6 @@
     <t>% of slaughtered</t>
   </si>
   <si>
-    <t>assumption. 2.3% for broilers</t>
-  </si>
-  <si>
     <t>Set to reach 5.0% for laying period. Avg gård A and B</t>
   </si>
   <si>
@@ -459,6 +453,24 @@
   </si>
   <si>
     <t>rapeseed cake for organic rations</t>
+  </si>
+  <si>
+    <t>5 mil. hatched, 0.5 mil dead during prod., 2.9 mil food, 0.6 mil pet food, 1.4 mil to destruction at slaughter</t>
+  </si>
+  <si>
+    <t>average_live_weight</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>https://lohmann-breeders.com/lohmanninfo/management-tools-to-influence-egg-weight-in-commercial-layers/</t>
+  </si>
+  <si>
+    <t>assumption to avoid too much organic poultry meat</t>
+  </si>
+  <si>
+    <t>SJV 2016-2020</t>
   </si>
 </sst>
 </file>
@@ -469,7 +481,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -544,6 +556,14 @@
     <font>
       <sz val="11"/>
       <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -719,11 +739,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -871,8 +892,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -1152,7 +1176,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q177"/>
+  <dimension ref="A1:Q180"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -1246,10 +1270,10 @@
         <v>4</v>
       </c>
       <c r="G5" s="79" t="s">
+        <v>118</v>
+      </c>
+      <c r="H5" t="s">
         <v>119</v>
-      </c>
-      <c r="H5" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -1318,7 +1342,7 @@
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E11" s="4"/>
       <c r="M11" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
@@ -1335,13 +1359,13 @@
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G12" s="79" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M12" s="80" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="N12" s="81"/>
       <c r="O12" s="81"/>
@@ -1366,13 +1390,13 @@
         <v>2</v>
       </c>
       <c r="F13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G13" s="79" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M13" s="83" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="N13" s="84"/>
       <c r="O13" s="84"/>
@@ -1395,10 +1419,10 @@
         <v>1.7</v>
       </c>
       <c r="F14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H14" t="s">
         <v>43</v>
@@ -1415,82 +1439,80 @@
         <v>3.45</v>
       </c>
       <c r="F15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G15" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
       <c r="D16" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="78">
+      <c r="E16" s="91">
+        <v>48</v>
+      </c>
+      <c r="F16" t="s">
+        <v>122</v>
+      </c>
+      <c r="G16" s="79" t="s">
+        <v>130</v>
+      </c>
+      <c r="H16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
         <v>5</v>
       </c>
-      <c r="F16" t="s">
-        <v>123</v>
-      </c>
-      <c r="G16" s="79" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E17" s="4"/>
+      <c r="E17" s="91">
+        <v>100</v>
+      </c>
+      <c r="F17" t="s">
+        <v>122</v>
+      </c>
+      <c r="G17" s="79" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="15"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="10"/>
-      <c r="D19" s="7" t="s">
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="15"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="D20" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="13">
-        <v>0</v>
-      </c>
-      <c r="F19" s="7" t="s">
+      <c r="E20" s="13">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="8"/>
-      <c r="D20" t="s">
-        <v>40</v>
-      </c>
-      <c r="E20" s="11">
-        <f>(22.5/64*52+20.2/58*52)/2</f>
-        <v>18.195797413793102</v>
-      </c>
-      <c r="F20" t="s">
-        <v>51</v>
-      </c>
-      <c r="G20" t="s">
-        <v>52</v>
-      </c>
-      <c r="H20" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1498,19 +1520,24 @@
         <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C21" s="8"/>
       <c r="D21" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="14">
-        <f>E20</f>
+      <c r="E21" s="11">
+        <f>(22.5/64*52+20.2/58*52)/2</f>
         <v>18.195797413793102</v>
       </c>
-      <c r="F21" s="14" t="str">
-        <f>F20</f>
-        <v>kg/head/year</v>
+      <c r="F21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21" t="s">
+        <v>52</v>
+      </c>
+      <c r="H21" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1518,14 +1545,14 @@
         <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C22" s="8"/>
       <c r="D22" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="14">
-        <f>E20</f>
+        <f>E21</f>
         <v>18.195797413793102</v>
       </c>
       <c r="F22" s="14" t="str">
@@ -1535,24 +1562,22 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" t="s">
         <v>40</v>
       </c>
-      <c r="E23" s="11">
-        <f>20/60*52</f>
-        <v>17.333333333333332</v>
-      </c>
-      <c r="F23" t="s">
-        <v>51</v>
-      </c>
-      <c r="H23" t="s">
-        <v>44</v>
+      <c r="E23" s="14">
+        <f>E21</f>
+        <v>18.195797413793102</v>
+      </c>
+      <c r="F23" s="14" t="str">
+        <f>F22</f>
+        <v>kg/head/year</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -1560,19 +1585,21 @@
         <v>42</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="14">
-        <f>E23</f>
+      <c r="E24" s="11">
+        <f>20/60*52</f>
         <v>17.333333333333332</v>
       </c>
-      <c r="F24" s="14" t="str">
-        <f>F23</f>
-        <v>kg/head/year</v>
+      <c r="F24" t="s">
+        <v>51</v>
+      </c>
+      <c r="H24" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -1580,14 +1607,14 @@
         <v>42</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="14">
-        <f>E23</f>
+        <f>E24</f>
         <v>17.333333333333332</v>
       </c>
       <c r="F25" s="14" t="str">
@@ -1596,103 +1623,118 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" t="s">
+        <v>49</v>
+      </c>
       <c r="C26" s="8"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
+      <c r="D26" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="14">
+        <f>E24</f>
+        <v>17.333333333333332</v>
+      </c>
+      <c r="F26" s="14" t="str">
+        <f>F25</f>
+        <v>kg/head/year</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
+      <c r="C27" s="8"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D28" t="s">
+      <c r="A28" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B29" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" t="s">
+        <v>131</v>
+      </c>
+      <c r="E29">
+        <f>1.2/2</f>
+        <v>0.6</v>
+      </c>
+      <c r="F29" t="s">
+        <v>132</v>
+      </c>
+      <c r="H29" s="92" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" t="s">
+        <v>131</v>
+      </c>
+      <c r="E30">
+        <v>1.4</v>
+      </c>
+      <c r="F30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D31" t="s">
+        <v>131</v>
+      </c>
+      <c r="E31">
+        <v>1.6</v>
+      </c>
+      <c r="F31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E32" s="8"/>
+      <c r="G32" s="8"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D33" t="s">
         <v>14</v>
       </c>
-      <c r="E28" s="8">
-        <v>0</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="E33" s="79">
+        <v>1.17</v>
+      </c>
+      <c r="F33" t="s">
         <v>15</v>
       </c>
-      <c r="G28" s="8" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E29" s="8"/>
-      <c r="G29" s="8"/>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E30" s="8"/>
-      <c r="G30" s="8"/>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+      <c r="G33" s="8"/>
+      <c r="H33" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="70" t="s">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="70" t="s">
         <v>107</v>
       </c>
-      <c r="G32" s="6"/>
-      <c r="H32" s="70" t="s">
+      <c r="G35" s="6"/>
+      <c r="H35" s="70" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" t="s">
-        <v>46</v>
-      </c>
-      <c r="D33" t="s">
-        <v>111</v>
-      </c>
-      <c r="E33" s="4">
-        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B33,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>14.427074999999999</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" t="s">
-        <v>47</v>
-      </c>
-      <c r="D34" t="s">
-        <v>111</v>
-      </c>
-      <c r="E34" s="4">
-        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B34,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>35.955136032867976</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" t="s">
-        <v>48</v>
-      </c>
-      <c r="D35" t="s">
-        <v>111</v>
-      </c>
-      <c r="E35" s="4">
-        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B35,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>31.729574287646834</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -1700,14 +1742,14 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
         <v>111</v>
       </c>
       <c r="E36" s="4">
         <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B36,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>36.30498550425397</v>
+        <v>14.427074999999999</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -1715,59 +1757,59 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="D37" t="s">
         <v>111</v>
       </c>
       <c r="E37" s="4">
         <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B37,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>36.235119047619044</v>
+        <v>35.955136032867976</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
+      </c>
+      <c r="D38" t="s">
+        <v>111</v>
+      </c>
+      <c r="E38" s="4">
+        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B38,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>31.729574287646834</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s">
         <v>111</v>
       </c>
       <c r="E39" s="4">
-        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B39,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>14.427074999999999</v>
+        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B39,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>36.30498550425397</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
         <v>111</v>
       </c>
       <c r="E40" s="4">
-        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B40,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>31.765466750719003</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>42</v>
-      </c>
-      <c r="B41" t="s">
-        <v>48</v>
-      </c>
-      <c r="D41" t="s">
-        <v>111</v>
-      </c>
-      <c r="E41" s="4">
-        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B41,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>34.907873896644638</v>
+        <f>INDEX('Feed rations'!$W$19:$AA$19,MATCH(B40,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>36.235119047619044</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1775,14 +1817,14 @@
         <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
         <v>111</v>
       </c>
       <c r="E42" s="4">
         <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B42,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>38.050281042570276</v>
+        <v>14.427074999999999</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1790,103 +1832,94 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="D43" t="s">
         <v>111</v>
       </c>
       <c r="E43" s="4">
         <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B43,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>31.765466750719003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>48</v>
+      </c>
+      <c r="D44" t="s">
+        <v>111</v>
+      </c>
+      <c r="E44" s="4">
+        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B44,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>34.907873896644638</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" t="s">
+        <v>49</v>
+      </c>
+      <c r="D45" t="s">
+        <v>111</v>
+      </c>
+      <c r="E45" s="4">
+        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B45,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>38.050281042570276</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46" t="s">
+        <v>89</v>
+      </c>
+      <c r="D46" t="s">
+        <v>111</v>
+      </c>
+      <c r="E46" s="4">
+        <f>INDEX('Feed rations'!$AB$19:$AF$19,MATCH(B46,'Feed rations'!$AB$4:$AF$4,0))</f>
         <v>36.235119047619044</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="70" t="s">
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="70" t="s">
         <v>109</v>
       </c>
-      <c r="G45" s="6"/>
-      <c r="H45" s="70" t="s">
+      <c r="G48" s="6"/>
+      <c r="H48" s="70" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="90" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="88"/>
-      <c r="B46" s="88"/>
-      <c r="C46" s="88"/>
-      <c r="D46" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="E46" s="13">
-        <v>0</v>
-      </c>
-      <c r="F46" s="89"/>
-      <c r="G46" s="7" t="s">
+    <row r="49" spans="1:8" s="90" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="88"/>
+      <c r="B49" s="88"/>
+      <c r="C49" s="88"/>
+      <c r="D49" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E49" s="13">
+        <v>0</v>
+      </c>
+      <c r="F49" s="89"/>
+      <c r="G49" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H46" s="89"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>41</v>
-      </c>
-      <c r="B47" t="s">
-        <v>46</v>
-      </c>
-      <c r="C47" t="s">
-        <v>17</v>
-      </c>
-      <c r="D47" t="s">
-        <v>112</v>
-      </c>
-      <c r="E47" s="4">
-        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C47,'Feed rations'!$V$5:$V$17,0),MATCH(B47,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>43.682112995233247</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>41</v>
-      </c>
-      <c r="B48" t="s">
-        <v>46</v>
-      </c>
-      <c r="C48" t="s">
-        <v>19</v>
-      </c>
-      <c r="D48" t="s">
-        <v>112</v>
-      </c>
-      <c r="E48" s="4">
-        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C48,'Feed rations'!$V$5:$V$17,0),MATCH(B48,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>2.6881300304758931</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>41</v>
-      </c>
-      <c r="B49" t="s">
-        <v>46</v>
-      </c>
-      <c r="C49" t="s">
-        <v>18</v>
-      </c>
-      <c r="D49" t="s">
-        <v>112</v>
-      </c>
-      <c r="E49" s="4">
-        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C49,'Feed rations'!$V$5:$V$17,0),MATCH(B49,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>16.800812690474331</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H49" s="89"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>41</v>
       </c>
@@ -1894,17 +1927,17 @@
         <v>46</v>
       </c>
       <c r="C50" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D50" t="s">
         <v>112</v>
       </c>
       <c r="E50" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C50,'Feed rations'!$V$5:$V$17,0),MATCH(B50,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>3.920189627777344</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+        <v>43.682112995233247</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>41</v>
       </c>
@@ -1912,17 +1945,17 @@
         <v>46</v>
       </c>
       <c r="C51" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D51" t="s">
         <v>112</v>
       </c>
       <c r="E51" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C51,'Feed rations'!$V$5:$V$17,0),MATCH(B51,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2.6881300304758931</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>41</v>
       </c>
@@ -1930,17 +1963,17 @@
         <v>46</v>
       </c>
       <c r="C52" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D52" t="s">
         <v>112</v>
       </c>
       <c r="E52" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C52,'Feed rations'!$V$5:$V$17,0),MATCH(B52,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+        <v>16.800812690474331</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>41</v>
       </c>
@@ -1948,17 +1981,17 @@
         <v>46</v>
       </c>
       <c r="C53" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D53" t="s">
         <v>112</v>
       </c>
       <c r="E53" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C53,'Feed rations'!$V$5:$V$17,0),MATCH(B53,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>27.048006043083014</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+        <v>3.920189627777344</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>41</v>
       </c>
@@ -1966,7 +1999,7 @@
         <v>46</v>
       </c>
       <c r="C54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D54" t="s">
         <v>112</v>
@@ -1976,7 +2009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>41</v>
       </c>
@@ -1984,7 +2017,7 @@
         <v>46</v>
       </c>
       <c r="C55" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D55" t="s">
         <v>112</v>
@@ -1994,7 +2027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>41</v>
       </c>
@@ -2002,17 +2035,17 @@
         <v>46</v>
       </c>
       <c r="C56" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D56" t="s">
         <v>112</v>
       </c>
       <c r="E56" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C56,'Feed rations'!$V$5:$V$17,0),MATCH(B56,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+        <v>27.048006043083014</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>41</v>
       </c>
@@ -2020,17 +2053,17 @@
         <v>46</v>
       </c>
       <c r="C57" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D57" t="s">
         <v>112</v>
       </c>
       <c r="E57" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C57,'Feed rations'!$V$5:$V$17,0),MATCH(B57,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>5.8607486129561623</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>41</v>
       </c>
@@ -2038,7 +2071,7 @@
         <v>46</v>
       </c>
       <c r="C58" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D58" t="s">
         <v>112</v>
@@ -2048,7 +2081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>41</v>
       </c>
@@ -2056,7 +2089,7 @@
         <v>46</v>
       </c>
       <c r="C59" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D59" t="s">
         <v>112</v>
@@ -2066,61 +2099,61 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>41</v>
       </c>
       <c r="B60" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C60" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D60" t="s">
         <v>112</v>
       </c>
       <c r="E60" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C60,'Feed rations'!$V$5:$V$17,0),MATCH(B60,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>52.05847593594973</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+        <v>5.8607486129561623</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>41</v>
       </c>
       <c r="B61" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C61" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D61" t="s">
         <v>112</v>
       </c>
       <c r="E61" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C61,'Feed rations'!$V$5:$V$17,0),MATCH(B61,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3440650152379465</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>41</v>
       </c>
       <c r="B62" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C62" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D62" t="s">
         <v>112</v>
       </c>
       <c r="E62" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C62,'Feed rations'!$V$5:$V$17,0),MATCH(B62,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>12.963626223585813</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>41</v>
       </c>
@@ -2128,17 +2161,17 @@
         <v>47</v>
       </c>
       <c r="C63" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D63" t="s">
         <v>112</v>
       </c>
       <c r="E63" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C63,'Feed rations'!$V$5:$V$17,0),MATCH(B63,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.960094813888672</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+        <v>52.05847593594973</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>41</v>
       </c>
@@ -2146,14 +2179,14 @@
         <v>47</v>
       </c>
       <c r="C64" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D64" t="s">
         <v>112</v>
       </c>
       <c r="E64" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C64,'Feed rations'!$V$5:$V$17,0),MATCH(B64,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3440650152379465</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -2164,14 +2197,14 @@
         <v>47</v>
       </c>
       <c r="C65" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D65" t="s">
         <v>112</v>
       </c>
       <c r="E65" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C65,'Feed rations'!$V$5:$V$17,0),MATCH(B65,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>12.963626223585813</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -2182,14 +2215,14 @@
         <v>47</v>
       </c>
       <c r="C66" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D66" t="s">
         <v>112</v>
       </c>
       <c r="E66" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C66,'Feed rations'!$V$5:$V$17,0),MATCH(B66,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>24.343208405260931</v>
+        <v>1.960094813888672</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -2200,7 +2233,7 @@
         <v>47</v>
       </c>
       <c r="C67" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D67" t="s">
         <v>112</v>
@@ -2218,14 +2251,14 @@
         <v>47</v>
       </c>
       <c r="C68" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D68" t="s">
         <v>112</v>
       </c>
       <c r="E68" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C68,'Feed rations'!$V$5:$V$17,0),MATCH(B68,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.7471204866054095</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -2236,14 +2269,14 @@
         <v>47</v>
       </c>
       <c r="C69" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D69" t="s">
         <v>112</v>
       </c>
       <c r="E69" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C69,'Feed rations'!$V$5:$V$17,0),MATCH(B69,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>24.343208405260931</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2254,14 +2287,14 @@
         <v>47</v>
       </c>
       <c r="C70" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D70" t="s">
         <v>112</v>
       </c>
       <c r="E70" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C70,'Feed rations'!$V$5:$V$17,0),MATCH(B70,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>5.5834091194714803</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -2272,14 +2305,14 @@
         <v>47</v>
       </c>
       <c r="C71" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D71" t="s">
         <v>112</v>
       </c>
       <c r="E71" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C71,'Feed rations'!$V$5:$V$17,0),MATCH(B71,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.7471204866054095</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2290,7 +2323,7 @@
         <v>47</v>
       </c>
       <c r="C72" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D72" t="s">
         <v>112</v>
@@ -2305,17 +2338,17 @@
         <v>41</v>
       </c>
       <c r="B73" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C73" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D73" t="s">
         <v>112</v>
       </c>
       <c r="E73" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C73,'Feed rations'!$V$5:$V$17,0),MATCH(B73,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>55.910178622144024</v>
+        <v>5.5834091194714803</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -2323,17 +2356,17 @@
         <v>41</v>
       </c>
       <c r="B74" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C74" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D74" t="s">
         <v>112</v>
       </c>
       <c r="E74" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C74,'Feed rations'!$V$5:$V$17,0),MATCH(B74,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3475047658841042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -2341,17 +2374,17 @@
         <v>41</v>
       </c>
       <c r="B75" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C75" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D75" t="s">
         <v>112</v>
       </c>
       <c r="E75" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C75,'Feed rations'!$V$5:$V$17,0),MATCH(B75,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>9.5448254250124034</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -2362,14 +2395,14 @@
         <v>48</v>
       </c>
       <c r="C76" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D76" t="s">
         <v>112</v>
       </c>
       <c r="E76" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C76,'Feed rations'!$V$5:$V$17,0),MATCH(B76,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>3.2003238189747476</v>
+        <v>55.910178622144024</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2380,14 +2413,14 @@
         <v>48</v>
       </c>
       <c r="C77" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D77" t="s">
         <v>112</v>
       </c>
       <c r="E77" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C77,'Feed rations'!$V$5:$V$17,0),MATCH(B77,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3475047658841042</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -2398,14 +2431,14 @@
         <v>48</v>
       </c>
       <c r="C78" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D78" t="s">
         <v>112</v>
       </c>
       <c r="E78" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C78,'Feed rations'!$V$5:$V$17,0),MATCH(B78,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>9.5448254250124034</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -2416,14 +2449,14 @@
         <v>48</v>
       </c>
       <c r="C79" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D79" t="s">
         <v>112</v>
       </c>
       <c r="E79" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C79,'Feed rations'!$V$5:$V$17,0),MATCH(B79,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>21.742772443376154</v>
+        <v>3.2003238189747476</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -2434,7 +2467,7 @@
         <v>48</v>
       </c>
       <c r="C80" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D80" t="s">
         <v>112</v>
@@ -2452,14 +2485,14 @@
         <v>48</v>
       </c>
       <c r="C81" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D81" t="s">
         <v>112</v>
       </c>
       <c r="E81" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C81,'Feed rations'!$V$5:$V$17,0),MATCH(B81,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3343217197924386</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -2470,14 +2503,14 @@
         <v>48</v>
       </c>
       <c r="C82" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D82" t="s">
         <v>112</v>
       </c>
       <c r="E82" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C82,'Feed rations'!$V$5:$V$17,0),MATCH(B82,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3788420860209438</v>
+        <v>21.742772443376154</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -2488,14 +2521,14 @@
         <v>48</v>
       </c>
       <c r="C83" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D83" t="s">
         <v>112</v>
       </c>
       <c r="E83" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C83,'Feed rations'!$V$5:$V$17,0),MATCH(B83,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>5.5412311187951762</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -2506,14 +2539,14 @@
         <v>48</v>
       </c>
       <c r="C84" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D84" t="s">
         <v>112</v>
       </c>
       <c r="E84" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C84,'Feed rations'!$V$5:$V$17,0),MATCH(B84,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3343217197924386</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -2524,14 +2557,14 @@
         <v>48</v>
       </c>
       <c r="C85" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D85" t="s">
         <v>112</v>
       </c>
       <c r="E85" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C85,'Feed rations'!$V$5:$V$17,0),MATCH(B85,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3788420860209438</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2539,17 +2572,17 @@
         <v>41</v>
       </c>
       <c r="B86" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C86" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D86" t="s">
         <v>112</v>
       </c>
       <c r="E86" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C86,'Feed rations'!$V$5:$V$17,0),MATCH(B86,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>58.797927209288808</v>
+        <v>5.5412311187951762</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2557,17 +2590,17 @@
         <v>41</v>
       </c>
       <c r="B87" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C87" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D87" t="s">
         <v>112</v>
       </c>
       <c r="E87" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C87,'Feed rations'!$V$5:$V$17,0),MATCH(B87,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3523075713499491</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -2575,17 +2608,17 @@
         <v>41</v>
       </c>
       <c r="B88" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C88" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D88" t="s">
         <v>112</v>
       </c>
       <c r="E88" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C88,'Feed rations'!$V$5:$V$17,0),MATCH(B88,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>8.4519223209371823</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -2596,14 +2629,14 @@
         <v>49</v>
       </c>
       <c r="C89" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D89" t="s">
         <v>112</v>
       </c>
       <c r="E89" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C89,'Feed rations'!$V$5:$V$17,0),MATCH(B89,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>2.1974998034436672</v>
+        <v>58.797927209288808</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -2614,14 +2647,14 @@
         <v>49</v>
       </c>
       <c r="C90" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D90" t="s">
         <v>112</v>
       </c>
       <c r="E90" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C90,'Feed rations'!$V$5:$V$17,0),MATCH(B90,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3523075713499491</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2632,14 +2665,14 @@
         <v>49</v>
       </c>
       <c r="C91" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D91" t="s">
         <v>112</v>
       </c>
       <c r="E91" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C91,'Feed rations'!$V$5:$V$17,0),MATCH(B91,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>8.4519223209371823</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -2650,14 +2683,14 @@
         <v>49</v>
       </c>
       <c r="C92" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D92" t="s">
         <v>112</v>
       </c>
       <c r="E92" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C92,'Feed rations'!$V$5:$V$17,0),MATCH(B92,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>19.824838165705017</v>
+        <v>2.1974998034436672</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -2668,7 +2701,7 @@
         <v>49</v>
       </c>
       <c r="C93" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D93" t="s">
         <v>112</v>
@@ -2686,14 +2719,14 @@
         <v>49</v>
       </c>
       <c r="C94" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D94" t="s">
         <v>112</v>
       </c>
       <c r="E94" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C94,'Feed rations'!$V$5:$V$17,0),MATCH(B94,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3343217197924386</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2704,14 +2737,14 @@
         <v>49</v>
       </c>
       <c r="C95" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D95" t="s">
         <v>112</v>
       </c>
       <c r="E95" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C95,'Feed rations'!$V$5:$V$17,0),MATCH(B95,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>2.8828262179940776</v>
+        <v>19.824838165705017</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -2722,14 +2755,14 @@
         <v>49</v>
       </c>
       <c r="C96" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D96" t="s">
         <v>112</v>
       </c>
       <c r="E96" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C96,'Feed rations'!$V$5:$V$17,0),MATCH(B96,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>5.1583569914888532</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
@@ -2740,14 +2773,14 @@
         <v>49</v>
       </c>
       <c r="C97" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D97" t="s">
         <v>112</v>
       </c>
       <c r="E97" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C97,'Feed rations'!$V$5:$V$17,0),MATCH(B97,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3343217197924386</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -2758,14 +2791,14 @@
         <v>49</v>
       </c>
       <c r="C98" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D98" t="s">
         <v>112</v>
       </c>
       <c r="E98" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C98,'Feed rations'!$V$5:$V$17,0),MATCH(B98,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>2.8828262179940776</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
@@ -2773,17 +2806,17 @@
         <v>41</v>
       </c>
       <c r="B99" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C99" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D99" t="s">
         <v>112</v>
       </c>
       <c r="E99" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C99,'Feed rations'!$V$5:$V$17,0),MATCH(B99,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>58.797927209288808</v>
+        <v>5.1583569914888532</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -2791,17 +2824,17 @@
         <v>41</v>
       </c>
       <c r="B100" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C100" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D100" t="s">
         <v>112</v>
       </c>
       <c r="E100" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C100,'Feed rations'!$V$5:$V$17,0),MATCH(B100,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3523075713499491</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
@@ -2809,17 +2842,17 @@
         <v>41</v>
       </c>
       <c r="B101" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C101" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D101" t="s">
         <v>112</v>
       </c>
       <c r="E101" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C101,'Feed rations'!$V$5:$V$17,0),MATCH(B101,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>8.4519223209371823</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
@@ -2830,14 +2863,14 @@
         <v>89</v>
       </c>
       <c r="C102" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D102" t="s">
         <v>112</v>
       </c>
       <c r="E102" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C102,'Feed rations'!$V$5:$V$17,0),MATCH(B102,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>2.1974998034436672</v>
+        <v>58.797927209288808</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -2848,14 +2881,14 @@
         <v>89</v>
       </c>
       <c r="C103" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D103" t="s">
         <v>112</v>
       </c>
       <c r="E103" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C103,'Feed rations'!$V$5:$V$17,0),MATCH(B103,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3523075713499491</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -2866,14 +2899,14 @@
         <v>89</v>
       </c>
       <c r="C104" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D104" t="s">
         <v>112</v>
       </c>
       <c r="E104" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C104,'Feed rations'!$V$5:$V$17,0),MATCH(B104,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>8.4519223209371823</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
@@ -2884,14 +2917,14 @@
         <v>89</v>
       </c>
       <c r="C105" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D105" t="s">
         <v>112</v>
       </c>
       <c r="E105" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C105,'Feed rations'!$V$5:$V$17,0),MATCH(B105,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>19.824838165705017</v>
+        <v>2.1974998034436672</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -2902,7 +2935,7 @@
         <v>89</v>
       </c>
       <c r="C106" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D106" t="s">
         <v>112</v>
@@ -2920,14 +2953,14 @@
         <v>89</v>
       </c>
       <c r="C107" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D107" t="s">
         <v>112</v>
       </c>
       <c r="E107" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C107,'Feed rations'!$V$5:$V$17,0),MATCH(B107,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>1.3343217197924386</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -2938,14 +2971,14 @@
         <v>89</v>
       </c>
       <c r="C108" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D108" t="s">
         <v>112</v>
       </c>
       <c r="E108" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C108,'Feed rations'!$V$5:$V$17,0),MATCH(B108,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>2.8828262179940776</v>
+        <v>19.824838165705017</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -2956,14 +2989,14 @@
         <v>89</v>
       </c>
       <c r="C109" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D109" t="s">
         <v>112</v>
       </c>
       <c r="E109" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C109,'Feed rations'!$V$5:$V$17,0),MATCH(B109,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>5.1583569914888532</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
@@ -2974,14 +3007,14 @@
         <v>89</v>
       </c>
       <c r="C110" t="s">
-        <v>92</v>
+        <v>22</v>
       </c>
       <c r="D110" t="s">
         <v>112</v>
       </c>
       <c r="E110" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C110,'Feed rations'!$V$5:$V$17,0),MATCH(B110,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>1.3343217197924386</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
@@ -2992,72 +3025,72 @@
         <v>89</v>
       </c>
       <c r="C111" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D111" t="s">
         <v>112</v>
       </c>
       <c r="E111" s="4">
         <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C111,'Feed rations'!$V$5:$V$17,0),MATCH(B111,'Feed rations'!$W$4:$AA$4,0))</f>
-        <v>0</v>
+        <v>2.8828262179940776</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E112" s="4"/>
+      <c r="A112" t="s">
+        <v>41</v>
+      </c>
+      <c r="B112" t="s">
+        <v>89</v>
+      </c>
+      <c r="C112" t="s">
+        <v>23</v>
+      </c>
+      <c r="D112" t="s">
+        <v>112</v>
+      </c>
+      <c r="E112" s="4">
+        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C112,'Feed rations'!$V$5:$V$17,0),MATCH(B112,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>5.1583569914888532</v>
+      </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B113" t="s">
-        <v>46</v>
+        <v>89</v>
       </c>
       <c r="C113" t="s">
-        <v>17</v>
+        <v>92</v>
       </c>
       <c r="D113" t="s">
         <v>112</v>
       </c>
       <c r="E113" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C113,'Feed rations'!$V$5:$V$17,0),MATCH(B113,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>43.682112995233247</v>
+        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C113,'Feed rations'!$V$5:$V$17,0),MATCH(B113,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B114" t="s">
-        <v>46</v>
+        <v>89</v>
       </c>
       <c r="C114" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D114" t="s">
         <v>112</v>
       </c>
       <c r="E114" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C114,'Feed rations'!$V$5:$V$17,0),MATCH(B114,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>2.6881300304758931</v>
+        <f>INDEX('Feed rations'!$W$5:$AA$17,MATCH(C114,'Feed rations'!$V$5:$V$17,0),MATCH(B114,'Feed rations'!$W$4:$AA$4,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>42</v>
-      </c>
-      <c r="B115" t="s">
-        <v>46</v>
-      </c>
-      <c r="C115" t="s">
-        <v>18</v>
-      </c>
-      <c r="D115" t="s">
-        <v>112</v>
-      </c>
-      <c r="E115" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C115,'Feed rations'!$V$5:$V$17,0),MATCH(B115,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>16.800812690474331</v>
-      </c>
+      <c r="E115" s="4"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
@@ -3067,14 +3100,14 @@
         <v>46</v>
       </c>
       <c r="C116" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D116" t="s">
         <v>112</v>
       </c>
       <c r="E116" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C116,'Feed rations'!$V$5:$V$17,0),MATCH(B116,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>3.920189627777344</v>
+        <v>43.682112995233247</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
@@ -3085,14 +3118,14 @@
         <v>46</v>
       </c>
       <c r="C117" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D117" t="s">
         <v>112</v>
       </c>
       <c r="E117" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C117,'Feed rations'!$V$5:$V$17,0),MATCH(B117,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>2.6881300304758931</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
@@ -3103,14 +3136,14 @@
         <v>46</v>
       </c>
       <c r="C118" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D118" t="s">
         <v>112</v>
       </c>
       <c r="E118" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C118,'Feed rations'!$V$5:$V$17,0),MATCH(B118,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>16.800812690474331</v>
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.25">
@@ -3121,14 +3154,14 @@
         <v>46</v>
       </c>
       <c r="C119" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D119" t="s">
         <v>112</v>
       </c>
       <c r="E119" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C119,'Feed rations'!$V$5:$V$17,0),MATCH(B119,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>27.048006043083014</v>
+        <v>3.920189627777344</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -3139,7 +3172,7 @@
         <v>46</v>
       </c>
       <c r="C120" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D120" t="s">
         <v>112</v>
@@ -3156,21 +3189,15 @@
       <c r="B121" t="s">
         <v>46</v>
       </c>
-      <c r="C121" s="87" t="s">
-        <v>130</v>
+      <c r="C121" t="s">
+        <v>20</v>
       </c>
       <c r="D121" t="s">
         <v>112</v>
       </c>
       <c r="E121" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H121,'Feed rations'!$V$5:$V$17,0),MATCH(B121,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G121" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="H121" t="s">
-        <v>22</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C121,'Feed rations'!$V$5:$V$17,0),MATCH(B121,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
@@ -3181,14 +3208,14 @@
         <v>46</v>
       </c>
       <c r="C122" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D122" t="s">
         <v>112</v>
       </c>
       <c r="E122" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C122,'Feed rations'!$V$5:$V$17,0),MATCH(B122,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>27.048006043083014</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.25">
@@ -3199,14 +3226,14 @@
         <v>46</v>
       </c>
       <c r="C123" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D123" t="s">
         <v>112</v>
       </c>
       <c r="E123" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C123,'Feed rations'!$V$5:$V$17,0),MATCH(B123,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>5.8607486129561623</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.25">
@@ -3216,15 +3243,21 @@
       <c r="B124" t="s">
         <v>46</v>
       </c>
-      <c r="C124" t="s">
-        <v>92</v>
+      <c r="C124" s="87" t="s">
+        <v>128</v>
       </c>
       <c r="D124" t="s">
         <v>112</v>
       </c>
       <c r="E124" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C124,'Feed rations'!$V$5:$V$17,0),MATCH(B124,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H124,'Feed rations'!$V$5:$V$17,0),MATCH(B124,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G124" s="87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H124" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.25">
@@ -3235,7 +3268,7 @@
         <v>46</v>
       </c>
       <c r="C125" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D125" t="s">
         <v>112</v>
@@ -3250,17 +3283,17 @@
         <v>42</v>
       </c>
       <c r="B126" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C126" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D126" t="s">
         <v>112</v>
       </c>
       <c r="E126" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C126,'Feed rations'!$V$5:$V$17,0),MATCH(B126,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>58.016195973989106</v>
+        <v>5.8607486129561623</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
@@ -3268,10 +3301,10 @@
         <v>42</v>
       </c>
       <c r="B127" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C127" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D127" t="s">
         <v>112</v>
@@ -3286,17 +3319,17 @@
         <v>42</v>
       </c>
       <c r="B128" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C128" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D128" t="s">
         <v>112</v>
       </c>
       <c r="E128" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C128,'Feed rations'!$V$5:$V$17,0),MATCH(B128,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>13.254201084237993</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
@@ -3307,14 +3340,14 @@
         <v>47</v>
       </c>
       <c r="C129" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D129" t="s">
         <v>112</v>
       </c>
       <c r="E129" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C129,'Feed rations'!$V$5:$V$17,0),MATCH(B129,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>5.1156565588286975</v>
+        <v>58.016195973989106</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.25">
@@ -3325,14 +3358,14 @@
         <v>47</v>
       </c>
       <c r="C130" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D130" t="s">
         <v>112</v>
       </c>
       <c r="E130" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C130,'Feed rations'!$V$5:$V$17,0),MATCH(B130,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>8.2737362949343645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
@@ -3343,14 +3376,14 @@
         <v>47</v>
       </c>
       <c r="C131" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D131" t="s">
         <v>112</v>
       </c>
       <c r="E131" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C131,'Feed rations'!$V$5:$V$17,0),MATCH(B131,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>3.6907353080344469</v>
+        <v>13.254201084237993</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.25">
@@ -3361,14 +3394,14 @@
         <v>47</v>
       </c>
       <c r="C132" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D132" t="s">
         <v>112</v>
       </c>
       <c r="E132" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C132,'Feed rations'!$V$5:$V$17,0),MATCH(B132,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>5.1156565588286975</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
@@ -3379,14 +3412,14 @@
         <v>47</v>
       </c>
       <c r="C133" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D133" t="s">
         <v>112</v>
       </c>
       <c r="E133" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C133,'Feed rations'!$V$5:$V$17,0),MATCH(B133,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>2.3523367897362411</v>
+        <v>8.2737362949343645</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
@@ -3396,21 +3429,15 @@
       <c r="B134" t="s">
         <v>47</v>
       </c>
-      <c r="C134" s="87" t="s">
-        <v>130</v>
+      <c r="C134" t="s">
+        <v>20</v>
       </c>
       <c r="D134" t="s">
         <v>112</v>
       </c>
       <c r="E134" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H134,'Feed rations'!$V$5:$V$17,0),MATCH(B134,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>1.5817437034433346</v>
-      </c>
-      <c r="G134" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="H134" t="s">
-        <v>22</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C134,'Feed rations'!$V$5:$V$17,0),MATCH(B134,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>3.6907353080344469</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
@@ -3421,7 +3448,7 @@
         <v>47</v>
       </c>
       <c r="C135" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D135" t="s">
         <v>112</v>
@@ -3439,14 +3466,14 @@
         <v>47</v>
       </c>
       <c r="C136" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D136" t="s">
         <v>112</v>
       </c>
       <c r="E136" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C136,'Feed rations'!$V$5:$V$17,0),MATCH(B136,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>2.3523367897362411</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.25">
@@ -3456,15 +3483,21 @@
       <c r="B137" t="s">
         <v>47</v>
       </c>
-      <c r="C137" t="s">
-        <v>92</v>
+      <c r="C137" s="87" t="s">
+        <v>128</v>
       </c>
       <c r="D137" t="s">
         <v>112</v>
       </c>
       <c r="E137" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C137,'Feed rations'!$V$5:$V$17,0),MATCH(B137,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>6.1512255133907452</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H137,'Feed rations'!$V$5:$V$17,0),MATCH(B137,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>1.5817437034433346</v>
+      </c>
+      <c r="G137" s="87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H137" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.25">
@@ -3475,14 +3508,14 @@
         <v>47</v>
       </c>
       <c r="C138" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D138" t="s">
         <v>112</v>
       </c>
       <c r="E138" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C138,'Feed rations'!$V$5:$V$17,0),MATCH(B138,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>1.5641687734050753</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
@@ -3490,17 +3523,17 @@
         <v>42</v>
       </c>
       <c r="B139" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C139" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D139" t="s">
         <v>112</v>
       </c>
       <c r="E139" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C139,'Feed rations'!$V$5:$V$17,0),MATCH(B139,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>57.806020490924027</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.25">
@@ -3508,17 +3541,17 @@
         <v>42</v>
       </c>
       <c r="B140" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C140" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D140" t="s">
         <v>112</v>
       </c>
       <c r="E140" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C140,'Feed rations'!$V$5:$V$17,0),MATCH(B140,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>6.1512255133907452</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.25">
@@ -3526,17 +3559,17 @@
         <v>42</v>
       </c>
       <c r="B141" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C141" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D141" t="s">
         <v>112</v>
       </c>
       <c r="E141" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C141,'Feed rations'!$V$5:$V$17,0),MATCH(B141,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>14.91384967080074</v>
+        <v>1.5641687734050753</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.25">
@@ -3547,14 +3580,14 @@
         <v>48</v>
       </c>
       <c r="C142" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D142" t="s">
         <v>112</v>
       </c>
       <c r="E142" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C142,'Feed rations'!$V$5:$V$17,0),MATCH(B142,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>8.3761840506164251</v>
+        <v>57.806020490924027</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.25">
@@ -3565,14 +3598,14 @@
         <v>48</v>
       </c>
       <c r="C143" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D143" t="s">
         <v>112</v>
       </c>
       <c r="E143" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C143,'Feed rations'!$V$5:$V$17,0),MATCH(B143,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>4.1368681474671822</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.25">
@@ -3583,14 +3616,14 @@
         <v>48</v>
       </c>
       <c r="C144" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D144" t="s">
         <v>112</v>
       </c>
       <c r="E144" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C144,'Feed rations'!$V$5:$V$17,0),MATCH(B144,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>4.021954820011894</v>
+        <v>14.91384967080074</v>
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.25">
@@ -3601,14 +3634,14 @@
         <v>48</v>
       </c>
       <c r="C145" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D145" t="s">
         <v>112</v>
       </c>
       <c r="E145" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C145,'Feed rations'!$V$5:$V$17,0),MATCH(B145,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>8.3761840506164251</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.25">
@@ -3619,39 +3652,32 @@
         <v>48</v>
       </c>
       <c r="C146" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D146" t="s">
         <v>112</v>
       </c>
       <c r="E146" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C146,'Feed rations'!$V$5:$V$17,0),MATCH(B146,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>2.3652615404978614</v>
+        <v>4.1368681474671822</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A147" s="79" t="s">
-        <v>42</v>
-      </c>
-      <c r="B147" s="79" t="s">
+      <c r="A147" t="s">
+        <v>42</v>
+      </c>
+      <c r="B147" t="s">
         <v>48</v>
       </c>
-      <c r="C147" s="87" t="s">
-        <v>130</v>
-      </c>
-      <c r="D147" s="79" t="s">
-        <v>112</v>
-      </c>
-      <c r="E147" s="78">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H147,'Feed rations'!$V$5:$V$17,0),MATCH(B147,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0.7908718517216673</v>
-      </c>
-      <c r="F147" s="87"/>
-      <c r="G147" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="H147" t="s">
-        <v>22</v>
+      <c r="C147" t="s">
+        <v>20</v>
+      </c>
+      <c r="D147" t="s">
+        <v>112</v>
+      </c>
+      <c r="E147" s="4">
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C147,'Feed rations'!$V$5:$V$17,0),MATCH(B147,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>4.021954820011894</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
@@ -3662,7 +3688,7 @@
         <v>48</v>
       </c>
       <c r="C148" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D148" t="s">
         <v>112</v>
@@ -3680,32 +3706,39 @@
         <v>48</v>
       </c>
       <c r="C149" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D149" t="s">
         <v>112</v>
       </c>
       <c r="E149" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C149,'Feed rations'!$V$5:$V$17,0),MATCH(B149,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>2.3652615404978614</v>
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>42</v>
-      </c>
-      <c r="B150" t="s">
+      <c r="A150" s="79" t="s">
+        <v>42</v>
+      </c>
+      <c r="B150" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="C150" t="s">
-        <v>92</v>
-      </c>
-      <c r="D150" t="s">
-        <v>112</v>
-      </c>
-      <c r="E150" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C150,'Feed rations'!$V$5:$V$17,0),MATCH(B150,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>6.8069050412576626</v>
+      <c r="C150" s="87" t="s">
+        <v>128</v>
+      </c>
+      <c r="D150" s="79" t="s">
+        <v>112</v>
+      </c>
+      <c r="E150" s="78">
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H150,'Feed rations'!$V$5:$V$17,0),MATCH(B150,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0.7908718517216673</v>
+      </c>
+      <c r="F150" s="87"/>
+      <c r="G150" s="87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H150" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
@@ -3716,14 +3749,14 @@
         <v>48</v>
       </c>
       <c r="C151" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D151" t="s">
         <v>112</v>
       </c>
       <c r="E151" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C151,'Feed rations'!$V$5:$V$17,0),MATCH(B151,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0.78208438670253766</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
@@ -3731,17 +3764,17 @@
         <v>42</v>
       </c>
       <c r="B152" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C152" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D152" t="s">
         <v>112</v>
       </c>
       <c r="E152" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C152,'Feed rations'!$V$5:$V$17,0),MATCH(B152,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>57.595845007858948</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.25">
@@ -3749,17 +3782,17 @@
         <v>42</v>
       </c>
       <c r="B153" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C153" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D153" t="s">
         <v>112</v>
       </c>
       <c r="E153" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C153,'Feed rations'!$V$5:$V$17,0),MATCH(B153,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>6.8069050412576626</v>
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
@@ -3767,17 +3800,17 @@
         <v>42</v>
       </c>
       <c r="B154" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C154" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D154" t="s">
         <v>112</v>
       </c>
       <c r="E154" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C154,'Feed rations'!$V$5:$V$17,0),MATCH(B154,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>16.573498257363489</v>
+        <v>0.78208438670253766</v>
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
@@ -3788,14 +3821,14 @@
         <v>49</v>
       </c>
       <c r="C155" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D155" t="s">
         <v>112</v>
       </c>
       <c r="E155" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C155,'Feed rations'!$V$5:$V$17,0),MATCH(B155,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>11.636711542404154</v>
+        <v>57.595845007858948</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.25">
@@ -3806,7 +3839,7 @@
         <v>49</v>
       </c>
       <c r="C156" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D156" t="s">
         <v>112</v>
@@ -3824,14 +3857,14 @@
         <v>49</v>
       </c>
       <c r="C157" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D157" t="s">
         <v>112</v>
       </c>
       <c r="E157" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C157,'Feed rations'!$V$5:$V$17,0),MATCH(B157,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>4.3531743319893401</v>
+        <v>16.573498257363489</v>
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.25">
@@ -3842,14 +3875,14 @@
         <v>49</v>
       </c>
       <c r="C158" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D158" t="s">
         <v>112</v>
       </c>
       <c r="E158" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C158,'Feed rations'!$V$5:$V$17,0),MATCH(B158,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>11.636711542404154</v>
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
@@ -3860,14 +3893,14 @@
         <v>49</v>
       </c>
       <c r="C159" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D159" t="s">
         <v>112</v>
       </c>
       <c r="E159" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C159,'Feed rations'!$V$5:$V$17,0),MATCH(B159,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>2.3781862912594818</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.25">
@@ -3877,21 +3910,15 @@
       <c r="B160" t="s">
         <v>49</v>
       </c>
-      <c r="C160" s="87" t="s">
-        <v>130</v>
+      <c r="C160" t="s">
+        <v>20</v>
       </c>
       <c r="D160" t="s">
         <v>112</v>
       </c>
       <c r="E160" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H160,'Feed rations'!$V$5:$V$17,0),MATCH(B160,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G160" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="H160" t="s">
-        <v>22</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C160,'Feed rations'!$V$5:$V$17,0),MATCH(B160,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>4.3531743319893401</v>
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.25">
@@ -3902,7 +3929,7 @@
         <v>49</v>
       </c>
       <c r="C161" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D161" t="s">
         <v>112</v>
@@ -3920,14 +3947,14 @@
         <v>49</v>
       </c>
       <c r="C162" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D162" t="s">
         <v>112</v>
       </c>
       <c r="E162" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C162,'Feed rations'!$V$5:$V$17,0),MATCH(B162,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>2.3781862912594818</v>
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.25">
@@ -3937,15 +3964,21 @@
       <c r="B163" t="s">
         <v>49</v>
       </c>
-      <c r="C163" t="s">
-        <v>92</v>
+      <c r="C163" s="87" t="s">
+        <v>128</v>
       </c>
       <c r="D163" t="s">
         <v>112</v>
       </c>
       <c r="E163" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C163,'Feed rations'!$V$5:$V$17,0),MATCH(B163,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>7.4625845691245809</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H163,'Feed rations'!$V$5:$V$17,0),MATCH(B163,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G163" s="87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H163" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.25">
@@ -3956,7 +3989,7 @@
         <v>49</v>
       </c>
       <c r="C164" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D164" t="s">
         <v>112</v>
@@ -3971,17 +4004,17 @@
         <v>42</v>
       </c>
       <c r="B165" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C165" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D165" t="s">
         <v>112</v>
       </c>
       <c r="E165" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C165,'Feed rations'!$V$5:$V$17,0),MATCH(B165,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>57.595845007858948</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.25">
@@ -3989,17 +4022,17 @@
         <v>42</v>
       </c>
       <c r="B166" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C166" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="D166" t="s">
         <v>112</v>
       </c>
       <c r="E166" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C166,'Feed rations'!$V$5:$V$17,0),MATCH(B166,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>7.4625845691245809</v>
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.25">
@@ -4007,17 +4040,17 @@
         <v>42</v>
       </c>
       <c r="B167" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="C167" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D167" t="s">
         <v>112</v>
       </c>
       <c r="E167" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C167,'Feed rations'!$V$5:$V$17,0),MATCH(B167,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>16.573498257363489</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.25">
@@ -4028,14 +4061,14 @@
         <v>89</v>
       </c>
       <c r="C168" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="D168" t="s">
         <v>112</v>
       </c>
       <c r="E168" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C168,'Feed rations'!$V$5:$V$17,0),MATCH(B168,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>11.636711542404154</v>
+        <v>57.595845007858948</v>
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.25">
@@ -4046,7 +4079,7 @@
         <v>89</v>
       </c>
       <c r="C169" t="s">
-        <v>82</v>
+        <v>19</v>
       </c>
       <c r="D169" t="s">
         <v>112</v>
@@ -4064,14 +4097,14 @@
         <v>89</v>
       </c>
       <c r="C170" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D170" t="s">
         <v>112</v>
       </c>
       <c r="E170" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C170,'Feed rations'!$V$5:$V$17,0),MATCH(B170,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>4.3531743319893401</v>
+        <v>16.573498257363489</v>
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.25">
@@ -4082,14 +4115,14 @@
         <v>89</v>
       </c>
       <c r="C171" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="D171" t="s">
         <v>112</v>
       </c>
       <c r="E171" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C171,'Feed rations'!$V$5:$V$17,0),MATCH(B171,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>11.636711542404154</v>
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.25">
@@ -4100,14 +4133,14 @@
         <v>89</v>
       </c>
       <c r="C172" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D172" t="s">
         <v>112</v>
       </c>
       <c r="E172" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C172,'Feed rations'!$V$5:$V$17,0),MATCH(B172,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>2.3781862912594818</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.25">
@@ -4117,21 +4150,15 @@
       <c r="B173" t="s">
         <v>89</v>
       </c>
-      <c r="C173" s="87" t="s">
-        <v>130</v>
+      <c r="C173" t="s">
+        <v>20</v>
       </c>
       <c r="D173" t="s">
         <v>112</v>
       </c>
       <c r="E173" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H173,'Feed rations'!$V$5:$V$17,0),MATCH(B173,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
-      </c>
-      <c r="G173" s="87" t="s">
-        <v>131</v>
-      </c>
-      <c r="H173" t="s">
-        <v>22</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C173,'Feed rations'!$V$5:$V$17,0),MATCH(B173,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>4.3531743319893401</v>
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.25">
@@ -4142,7 +4169,7 @@
         <v>89</v>
       </c>
       <c r="C174" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D174" t="s">
         <v>112</v>
@@ -4160,14 +4187,14 @@
         <v>89</v>
       </c>
       <c r="C175" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="D175" t="s">
         <v>112</v>
       </c>
       <c r="E175" s="4">
         <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C175,'Feed rations'!$V$5:$V$17,0),MATCH(B175,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>0</v>
+        <v>2.3781862912594818</v>
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.25">
@@ -4177,15 +4204,21 @@
       <c r="B176" t="s">
         <v>89</v>
       </c>
-      <c r="C176" t="s">
-        <v>92</v>
+      <c r="C176" s="87" t="s">
+        <v>128</v>
       </c>
       <c r="D176" t="s">
         <v>112</v>
       </c>
       <c r="E176" s="4">
-        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C176,'Feed rations'!$V$5:$V$17,0),MATCH(B176,'Feed rations'!$AB$4:$AF$4,0))</f>
-        <v>7.4625845691245809</v>
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(H176,'Feed rations'!$V$5:$V$17,0),MATCH(B176,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G176" s="87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H176" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
@@ -4196,7 +4229,7 @@
         <v>89</v>
       </c>
       <c r="C177" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="D177" t="s">
         <v>112</v>
@@ -4206,9 +4239,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>42</v>
+      </c>
+      <c r="B178" t="s">
+        <v>89</v>
+      </c>
+      <c r="C178" t="s">
+        <v>23</v>
+      </c>
+      <c r="D178" t="s">
+        <v>112</v>
+      </c>
+      <c r="E178" s="4">
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C178,'Feed rations'!$V$5:$V$17,0),MATCH(B178,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>42</v>
+      </c>
+      <c r="B179" t="s">
+        <v>89</v>
+      </c>
+      <c r="C179" t="s">
+        <v>92</v>
+      </c>
+      <c r="D179" t="s">
+        <v>112</v>
+      </c>
+      <c r="E179" s="4">
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C179,'Feed rations'!$V$5:$V$17,0),MATCH(B179,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>7.4625845691245809</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>42</v>
+      </c>
+      <c r="B180" t="s">
+        <v>89</v>
+      </c>
+      <c r="C180" t="s">
+        <v>27</v>
+      </c>
+      <c r="D180" t="s">
+        <v>112</v>
+      </c>
+      <c r="E180" s="4">
+        <f>INDEX('Feed rations'!$AB$5:$AF$17,MATCH(C180,'Feed rations'!$V$5:$V$17,0),MATCH(B180,'Feed rations'!$AB$4:$AF$4,0))</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H29" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4249,14 +4339,14 @@
         <v>67</v>
       </c>
       <c r="F2" s="52" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G2" s="53"/>
       <c r="H2" s="53"/>
       <c r="I2" s="53"/>
       <c r="J2" s="53"/>
       <c r="K2" s="62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L2" s="55"/>
       <c r="M2" s="21"/>
@@ -6282,12 +6372,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>